<commit_message>
Mise à jour du dashboard Excel et ajout du rapport d'analyse
</commit_message>
<xml_diff>
--- a/excel/base_cliniques.xlsx
+++ b/excel/base_cliniques.xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\projet-analyse-cliniques\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\projet-analyse-cliniques\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A84FBF2-A797-4C6E-BFF0-92CAC2877843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB45F4D8-AF8F-454A-803A-43290D529879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Filtrage données " sheetId="17" r:id="rId1"/>
@@ -310,11 +310,11 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -396,10 +396,30 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:r>
-              <a:rPr lang="fr-FR" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
-              <a:t>Évolution mensuelle du nombre de patients  2026</a:t>
-            </a:r>
+            <a:endParaRPr lang="fr-FR" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
             <a:endParaRPr lang="en-US" sz="1200" b="1"/>
           </a:p>
         </c:rich>
@@ -19911,7 +19931,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4AA35906-9AF0-4EB8-AA1C-163F9A710BB6}" name="Tableau croisé dynamique1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Établissement">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4AA35906-9AF0-4EB8-AA1C-163F9A710BB6}" name="Tableau croisé dynamique1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Établissement">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -20000,7 +20020,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{894440FF-CFFC-43B7-BA96-FAB81D722703}" name="Tableau croisé dynamique10" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Département">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{894440FF-CFFC-43B7-BA96-FAB81D722703}" name="Tableau croisé dynamique10" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Département">
   <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -20089,7 +20109,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D8F800A4-C9F2-4999-BE01-ACC7975DF2E6}" name="Tableau croisé dynamique12" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="établissement" colHeaderCaption="activité">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D8F800A4-C9F2-4999-BE01-ACC7975DF2E6}" name="Tableau croisé dynamique12" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="établissement" colHeaderCaption="activité">
   <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -20313,7 +20333,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{397C8953-90D1-4D62-8330-93E5369FB4F9}" name="Tableau croisé dynamique15" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13" rowHeaderCaption="Mois">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{397C8953-90D1-4D62-8330-93E5369FB4F9}" name="Tableau croisé dynamique15" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="19" rowHeaderCaption="Mois">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -20784,22 +20804,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
@@ -30369,15 +30389,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
       <c r="H1" s="11"/>
       <c r="I1" s="11"/>
       <c r="J1" s="11"/>
@@ -30389,13 +30409,13 @@
       <c r="P1" s="9"/>
     </row>
     <row r="2" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
       <c r="H2" s="11"/>
       <c r="I2" s="11"/>
       <c r="J2" s="11"/>

</xml_diff>